<commit_message>
feat: trang Khách list/detail, đồng bộ liên hệ và prefetch
Tách #/customers khỏi modal, hợp nhất SĐT/MST/email/địa chỉ với shipper mặc định, sửa hydrate/clear sync và import Excel 10 cột.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/customer/customs_ops.xlsx
+++ b/public/templates/customer/customs_ops.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30309"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BB465D-D2A2-46DE-BAFB-430EF55A4987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E640FC6A-B44B-4D2F-B011-2FD121780627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50" yWindow="-50" windowWidth="38500" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19170" yWindow="0" windowWidth="19260" windowHeight="20910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Customers" sheetId="1" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="160">
   <si>
     <t>Prefix</t>
   </si>
@@ -29,29 +30,479 @@
     <t>Short Code</t>
   </si>
   <si>
-    <t>GLO</t>
+    <t>Tax Code</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Default Rate</t>
+  </si>
+  <si>
+    <t>Customer Type</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Global Forwarding Vietnam Co., Ltd</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>ABC000001</t>
-  </si>
-  <si>
-    <t>ABC Trading &amp; Export JSC</t>
+    <t>HƯỚNG DẪN IMPORT / ĐỒNG BỘ KHÁCH HÀNG</t>
+  </si>
+  <si>
+    <t>1. Không đổi tên cột ở sheet 'Import Customers'.</t>
+  </si>
+  <si>
+    <t>2. Customer Name: bắt buộc.</t>
+  </si>
+  <si>
+    <t>3. Customer Code (VD: GLO000001): khóa đồng bộ. Có mã đã tồn tại → cập nhật thông tin. Có mã chưa tồn tại → tạo mới với đúng mã đó.</t>
+  </si>
+  <si>
+    <t>4. Prefix (2-5 chữ A-Z): bắt buộc khi tạo mới. Khi cập nhật phải khớp prefix hiện có (không được đổi).</t>
+  </si>
+  <si>
+    <t>5. Nếu bỏ trống Customer Code: hệ thống tạo mới và tự sinh mã từ Prefix.</t>
+  </si>
+  <si>
+    <t>6. Short Code: tối đa 10 ký tự, tùy chọn.</t>
+  </si>
+  <si>
+    <t>7. Default Rate: đơn giá cố định VND/kg (có thể để trống).</t>
+  </si>
+  <si>
+    <t>8. Customer Type: FORWARDER | DIRECT_SHIPPER | AGENT | OTHER (mặc định DIRECT_SHIPPER).</t>
+  </si>
+  <si>
+    <t>9. Prefix và Customer Code sau khi tạo không thể đổi qua import.</t>
+  </si>
+  <si>
+    <t>DTE</t>
+  </si>
+  <si>
+    <t>DTE000001</t>
+  </si>
+  <si>
+    <t>ĐỨC THẮNG EXPRESS</t>
+  </si>
+  <si>
+    <t>ĐỨC THẮNG</t>
+  </si>
+  <si>
+    <t>HTS</t>
+  </si>
+  <si>
+    <t>HTS000002</t>
+  </si>
+  <si>
+    <t>HTS EXPRESS</t>
+  </si>
+  <si>
+    <t>MKL</t>
+  </si>
+  <si>
+    <t>MKL000003</t>
+  </si>
+  <si>
+    <t>MINH KHANG LOGISTICS</t>
+  </si>
+  <si>
+    <t>MINH KHANG</t>
+  </si>
+  <si>
+    <t>CCE</t>
+  </si>
+  <si>
+    <t>CCE000004</t>
+  </si>
+  <si>
+    <t>CÔNG CHÚA EXPRESS</t>
+  </si>
+  <si>
+    <t>CÔNG CHÚA</t>
+  </si>
+  <si>
+    <t>PCS</t>
+  </si>
+  <si>
+    <t>PCS000005</t>
+  </si>
+  <si>
+    <t>PCS LOGISTICS</t>
+  </si>
+  <si>
+    <t>TTP</t>
+  </si>
+  <si>
+    <t>TTP000006</t>
+  </si>
+  <si>
+    <t>TRƯỜNG THIÊN PHÚ</t>
+  </si>
+  <si>
+    <t>JER</t>
+  </si>
+  <si>
+    <t>JER000007</t>
+  </si>
+  <si>
+    <t>JER EXPRESS</t>
+  </si>
+  <si>
+    <t>VCA</t>
+  </si>
+  <si>
+    <t>VIETNCA EXPRESS</t>
+  </si>
+  <si>
+    <t>VIETNCA</t>
+  </si>
+  <si>
+    <t>VAU</t>
+  </si>
+  <si>
+    <t>VAU000009</t>
+  </si>
+  <si>
+    <t>VCA000008</t>
+  </si>
+  <si>
+    <t>VAU EXPRESS</t>
+  </si>
+  <si>
+    <t>ATU</t>
+  </si>
+  <si>
+    <t>ATU000010</t>
+  </si>
+  <si>
+    <t>TÚ BÉO</t>
+  </si>
+  <si>
+    <t>A TÚ</t>
+  </si>
+  <si>
+    <t>TPE</t>
+  </si>
+  <si>
+    <t>TPE000011</t>
+  </si>
+  <si>
+    <t>TÍN PHÁT EXPRESS</t>
+  </si>
+  <si>
+    <t>TÍN PHÁT</t>
+  </si>
+  <si>
+    <t>VIC</t>
+  </si>
+  <si>
+    <t>VIC000012</t>
+  </si>
+  <si>
+    <t>VICTORIA EXPRESS</t>
+  </si>
+  <si>
+    <t>TNL</t>
+  </si>
+  <si>
+    <t>TNL000013</t>
+  </si>
+  <si>
+    <t>TAM NHẬT LONG</t>
+  </si>
+  <si>
+    <t>TLE</t>
+  </si>
+  <si>
+    <t>TLE000014</t>
+  </si>
+  <si>
+    <t>THẾ LONG EXPRESS</t>
+  </si>
+  <si>
+    <t>THẾ LONG</t>
+  </si>
+  <si>
+    <t>TTE</t>
+  </si>
+  <si>
+    <t>TTE000015</t>
+  </si>
+  <si>
+    <t>THANH TÂM EXPRESS</t>
+  </si>
+  <si>
+    <t>THANH TÂM</t>
+  </si>
+  <si>
+    <t>SNE</t>
+  </si>
+  <si>
+    <t>SNE000016</t>
+  </si>
+  <si>
+    <t>SUNNY CDG</t>
+  </si>
+  <si>
+    <t>SNL</t>
+  </si>
+  <si>
+    <t>SNL000017</t>
+  </si>
+  <si>
+    <t>SUNNY LHR</t>
+  </si>
+  <si>
+    <t>SKY</t>
+  </si>
+  <si>
+    <t>SKY000018</t>
+  </si>
+  <si>
+    <t>SKYLINK</t>
+  </si>
+  <si>
+    <t>SKYLINK EXPRESS</t>
+  </si>
+  <si>
+    <t>QNE</t>
+  </si>
+  <si>
+    <t>QNE000019</t>
+  </si>
+  <si>
+    <t>QUÝ NAM EXPRESS</t>
+  </si>
+  <si>
+    <t>QUÝ NAM</t>
+  </si>
+  <si>
+    <t>PTL</t>
+  </si>
+  <si>
+    <t>PTL000020</t>
+  </si>
+  <si>
+    <t>PHÁT TÀI LOGISTICS</t>
+  </si>
+  <si>
+    <t>PHÁT TÀI</t>
+  </si>
+  <si>
+    <t>PRM</t>
+  </si>
+  <si>
+    <t>PRM000021</t>
+  </si>
+  <si>
+    <t>PARAMOUNT</t>
+  </si>
+  <si>
+    <t>PARAMOUNT LOGISTICS</t>
+  </si>
+  <si>
+    <t>NST</t>
+  </si>
+  <si>
+    <t>NST000022</t>
+  </si>
+  <si>
+    <t>NISI TRẦN HỒ</t>
+  </si>
+  <si>
+    <t>BI</t>
+  </si>
+  <si>
+    <t>YUE</t>
+  </si>
+  <si>
+    <t>YUE000023</t>
+  </si>
+  <si>
+    <t>YU EXPRESS</t>
+  </si>
+  <si>
+    <t>NHU</t>
+  </si>
+  <si>
+    <t>NSK</t>
+  </si>
+  <si>
+    <t>NSK000024</t>
+  </si>
+  <si>
+    <t>NEWSKY EXPRESS</t>
+  </si>
+  <si>
+    <t>NEWSKY</t>
+  </si>
+  <si>
+    <t>NAE</t>
+  </si>
+  <si>
+    <t>NAE000025</t>
+  </si>
+  <si>
+    <t>NAM ANH EXPRESS</t>
+  </si>
+  <si>
+    <t>NAM ANH</t>
+  </si>
+  <si>
+    <t>MKE</t>
+  </si>
+  <si>
+    <t>MKE000026</t>
+  </si>
+  <si>
+    <t>MINH KHÔI EXPRESS</t>
+  </si>
+  <si>
+    <t>MINH KHÔI</t>
+  </si>
+  <si>
+    <t>LTE</t>
+  </si>
+  <si>
+    <t>LTE000027</t>
+  </si>
+  <si>
+    <t>LITA EXPRESS</t>
+  </si>
+  <si>
+    <t>LITA</t>
+  </si>
+  <si>
+    <t>LNE</t>
+  </si>
+  <si>
+    <t>LNE000028</t>
+  </si>
+  <si>
+    <t>LINO EXPRESS</t>
+  </si>
+  <si>
+    <t>LINO</t>
+  </si>
+  <si>
+    <t>SPX</t>
+  </si>
+  <si>
+    <t>SPX000029</t>
+  </si>
+  <si>
+    <t>SHOPEE</t>
+  </si>
+  <si>
+    <t>SHOPEE EXPRESS</t>
+  </si>
+  <si>
+    <t>GSE</t>
+  </si>
+  <si>
+    <t>GSE000030</t>
+  </si>
+  <si>
+    <t>GSHIP EXPRESS</t>
+  </si>
+  <si>
+    <t>GSHIP</t>
+  </si>
+  <si>
+    <t>GPE</t>
+  </si>
+  <si>
+    <t>GPE000031</t>
+  </si>
+  <si>
+    <t>GIA PHÚ</t>
+  </si>
+  <si>
+    <t>GWE</t>
+  </si>
+  <si>
+    <t>GWE000032</t>
+  </si>
+  <si>
+    <t>GATEWAY</t>
+  </si>
+  <si>
+    <t>GATEWAY EXPRESS</t>
+  </si>
+  <si>
+    <t>ELO</t>
+  </si>
+  <si>
+    <t>ELO000033</t>
+  </si>
+  <si>
+    <t>ELOG LOGISTICS</t>
+  </si>
+  <si>
+    <t>ELOG</t>
+  </si>
+  <si>
+    <t>CYL</t>
+  </si>
+  <si>
+    <t>CYL000034</t>
+  </si>
+  <si>
+    <t>CYL EXPRESS</t>
+  </si>
+  <si>
+    <t>CTE</t>
+  </si>
+  <si>
+    <t>CTE000035</t>
+  </si>
+  <si>
+    <t>CT EXPRESS</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>CTL</t>
+  </si>
+  <si>
+    <t>CTL000036</t>
+  </si>
+  <si>
+    <t>CITYLINK EXPRESS</t>
+  </si>
+  <si>
+    <t>CITYLINK</t>
+  </si>
+  <si>
+    <t>CGK</t>
+  </si>
+  <si>
+    <t>CGK000037</t>
+  </si>
+  <si>
+    <t>MR JUNG</t>
+  </si>
+  <si>
+    <t>MRP</t>
+  </si>
+  <si>
+    <t>MRP000038</t>
+  </si>
+  <si>
+    <t>MR PHI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,6 +515,17 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -91,11 +553,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -435,13 +898,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="4" width="18" customWidth="1"/>
+    <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -454,33 +917,640 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B29" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D29" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>124</v>
+      </c>
+      <c r="B30" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" t="s">
+        <v>133</v>
+      </c>
+      <c r="C32" t="s">
+        <v>134</v>
+      </c>
+      <c r="D32" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>135</v>
+      </c>
+      <c r="B33" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>139</v>
+      </c>
+      <c r="B34" t="s">
+        <v>140</v>
+      </c>
+      <c r="C34" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" t="s">
+        <v>144</v>
+      </c>
+      <c r="C35" t="s">
+        <v>145</v>
+      </c>
+      <c r="D35" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>146</v>
+      </c>
+      <c r="B36" t="s">
+        <v>147</v>
+      </c>
+      <c r="C36" t="s">
+        <v>148</v>
+      </c>
+      <c r="D36" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>150</v>
+      </c>
+      <c r="B37" t="s">
+        <v>151</v>
+      </c>
+      <c r="C37" t="s">
+        <v>152</v>
+      </c>
+      <c r="D37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>154</v>
+      </c>
+      <c r="B38" t="s">
+        <v>155</v>
+      </c>
+      <c r="C38" t="s">
+        <v>156</v>
+      </c>
+      <c r="D38" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>157</v>
+      </c>
+      <c r="B39" t="s">
+        <v>158</v>
+      </c>
+      <c r="C39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D39" t="s">
+        <v>159</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="17" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>